<commit_message>
Updated Documentation files. Updated MCU symbol
</commit_message>
<xml_diff>
--- a/Documentation/cAiGED_STM32N657X0H3Q_VFBGA264_Pin_Assignment.xlsx
+++ b/Documentation/cAiGED_STM32N657X0H3Q_VFBGA264_Pin_Assignment.xlsx
@@ -8,17 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daniel.silva\Documents\Documentos Daniel\Altium Projects - D\cAiGED\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC77671E-9C4D-47BF-A44F-E2568A6CA5D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9C310D-74B8-435D-9F37-D7F3F7E48A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-16425" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-16425" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="Essential Pins" sheetId="2" r:id="rId2"/>
-    <sheet name="Power &amp; Ground" sheetId="3" r:id="rId3"/>
-    <sheet name="Deferred Interfaces" sheetId="4" r:id="rId4"/>
-    <sheet name="Sources" sheetId="5" r:id="rId5"/>
+    <sheet name="Sources" sheetId="5" r:id="rId2"/>
+    <sheet name="Essential Pins" sheetId="2" r:id="rId3"/>
+    <sheet name="Power &amp; Ground" sheetId="3" r:id="rId4"/>
+    <sheet name="Deferred Interfaces" sheetId="4" r:id="rId5"/>
+    <sheet name="Gigabit Ethernet" sheetId="6" r:id="rId6"/>
+    <sheet name="Connector Support" sheetId="7" r:id="rId7"/>
+    <sheet name="USB" sheetId="8" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Connector Support'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Gigabit Ethernet'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">USB!$A$1:$H$11</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -29,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="481">
   <si>
     <t>cAiGED STM32N657X0H3Q VFBGA264 Pin Assignment Baseline</t>
   </si>
@@ -1013,6 +1021,465 @@
   </si>
   <si>
     <t>https://www.st.com/resource/en/datasheet/stm32n657x0.pdf</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18; STM32N6570-DK uses PD3</t>
+  </si>
+  <si>
+    <t>PHY interrupt</t>
+  </si>
+  <si>
+    <t>ETH1_PHY_INTN</t>
+  </si>
+  <si>
+    <t>ETH_MDINT</t>
+  </si>
+  <si>
+    <t>PD3</t>
+  </si>
+  <si>
+    <t>E13</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18; STM32N6570-DK uses PD12</t>
+  </si>
+  <si>
+    <t>PHY management data</t>
+  </si>
+  <si>
+    <t>ETH1_MDIO</t>
+  </si>
+  <si>
+    <t>ETH_MDIO</t>
+  </si>
+  <si>
+    <t>PD12</t>
+  </si>
+  <si>
+    <t>C13</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18; STM32N6570-DK uses PD1</t>
+  </si>
+  <si>
+    <t>PHY management clock</t>
+  </si>
+  <si>
+    <t>ETH1_MDC</t>
+  </si>
+  <si>
+    <t>ETH_MDC</t>
+  </si>
+  <si>
+    <t>PD1</t>
+  </si>
+  <si>
+    <t>A14</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18/20</t>
+  </si>
+  <si>
+    <t>RGMII TXD3</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_TXD3</t>
+  </si>
+  <si>
+    <t>ETH_TXD3</t>
+  </si>
+  <si>
+    <t>PG4</t>
+  </si>
+  <si>
+    <t>RGMII TXD2</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_TXD2</t>
+  </si>
+  <si>
+    <t>ETH_TXD2</t>
+  </si>
+  <si>
+    <t>PG3</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>RGMII RXD1</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_RXD1</t>
+  </si>
+  <si>
+    <t>ETH_RXD1</t>
+  </si>
+  <si>
+    <t>PF15</t>
+  </si>
+  <si>
+    <t>N1</t>
+  </si>
+  <si>
+    <t>RGMII RXD0</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_RXD0</t>
+  </si>
+  <si>
+    <t>ETH_RXD0</t>
+  </si>
+  <si>
+    <t>PF14</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>RGMII TXD1</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_TXD1</t>
+  </si>
+  <si>
+    <t>ETH_TXD1</t>
+  </si>
+  <si>
+    <t>PF13</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>RGMII TXD0</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_TXD0</t>
+  </si>
+  <si>
+    <t>ETH_TXD0</t>
+  </si>
+  <si>
+    <t>PF12</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>RGMII TX control</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_TX_CTL</t>
+  </si>
+  <si>
+    <t>ETH_TX_CTL</t>
+  </si>
+  <si>
+    <t>PF11</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>RGMII RX control</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_RX_CTL</t>
+  </si>
+  <si>
+    <t>ETH_RX_CTL</t>
+  </si>
+  <si>
+    <t>PF10</t>
+  </si>
+  <si>
+    <t>L4</t>
+  </si>
+  <si>
+    <t>RGMII RXD3</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_RXD3</t>
+  </si>
+  <si>
+    <t>ETH_RXD3</t>
+  </si>
+  <si>
+    <t>PF9</t>
+  </si>
+  <si>
+    <t>RGMII RXD2</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_RXD2</t>
+  </si>
+  <si>
+    <t>ETH_RXD2</t>
+  </si>
+  <si>
+    <t>PF8</t>
+  </si>
+  <si>
+    <t>N3</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18/20; STM32N6570-DK</t>
+  </si>
+  <si>
+    <t>RGMII RX clock</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_RX_CLK</t>
+  </si>
+  <si>
+    <t>ETH_RX_CLK</t>
+  </si>
+  <si>
+    <t>PF7</t>
+  </si>
+  <si>
+    <t>M1</t>
+  </si>
+  <si>
+    <t>125 MHz Ethernet clock</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_CLK125</t>
+  </si>
+  <si>
+    <t>ETH_CLK125</t>
+  </si>
+  <si>
+    <t>PF2</t>
+  </si>
+  <si>
+    <t>M2</t>
+  </si>
+  <si>
+    <t>RGMII TX clock</t>
+  </si>
+  <si>
+    <t>ETH1_RGMII_GTX_CLK</t>
+  </si>
+  <si>
+    <t>ETH_GTX_CLK</t>
+  </si>
+  <si>
+    <t>PF0</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>Reference / Notes</t>
+  </si>
+  <si>
+    <t>Ethernet Function</t>
+  </si>
+  <si>
+    <t>Second port optional but pins reserved</t>
+  </si>
+  <si>
+    <t>VBUS power switch if host, ESD, connector-specific ID/CC implementation</t>
+  </si>
+  <si>
+    <t>OTG2_HSDP/HSDM</t>
+  </si>
+  <si>
+    <t>USB Type-A host or USB Type-C</t>
+  </si>
+  <si>
+    <t>USB2</t>
+  </si>
+  <si>
+    <t>Preferred user USB port</t>
+  </si>
+  <si>
+    <t>VBUS ESD/OVP, current/power switch as required, Type-C CC network/PD handling, connector shield strategy</t>
+  </si>
+  <si>
+    <t>OTG1_HSDP/HSDM + UCPD1_CC1/CC2</t>
+  </si>
+  <si>
+    <t>USB Type-C</t>
+  </si>
+  <si>
+    <t>USB1</t>
+  </si>
+  <si>
+    <t>Architecture selected; PHY TBD</t>
+  </si>
+  <si>
+    <t>Gigabit PHY, 25 MHz PHY clock/crystal as required, magnetics, RGMII termination/delay network, ESD, PHY reset</t>
+  </si>
+  <si>
+    <t>15 RGMII/management signals + optional PHY INT</t>
+  </si>
+  <si>
+    <t>RJ45 with integrated magnetics or RJ45 + external magnetics</t>
+  </si>
+  <si>
+    <t>Gigabit Ethernet</t>
+  </si>
+  <si>
+    <t>Design status</t>
+  </si>
+  <si>
+    <t>Required external circuitry</t>
+  </si>
+  <si>
+    <t>MCU signals</t>
+  </si>
+  <si>
+    <t>Connector choice</t>
+  </si>
+  <si>
+    <t>Interface</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18</t>
+  </si>
+  <si>
+    <t>Needed only for connector/OTG architecture</t>
+  </si>
+  <si>
+    <t>OTG ID</t>
+  </si>
+  <si>
+    <t>USB2_ID</t>
+  </si>
+  <si>
+    <t>OTG2_ID</t>
+  </si>
+  <si>
+    <t>E6</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18; USB PHY characteristics</t>
+  </si>
+  <si>
+    <t>200 Ω external resistor to GND per USB PHY requirement</t>
+  </si>
+  <si>
+    <t>USB PHY tuning</t>
+  </si>
+  <si>
+    <t>USB2_TXRTUNE</t>
+  </si>
+  <si>
+    <t>OTG2_TXRTUNE</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>DS14791 Table 18; VFBGA264</t>
+  </si>
+  <si>
+    <t>Second USB port</t>
+  </si>
+  <si>
+    <t>USB2 HS/FS D+</t>
+  </si>
+  <si>
+    <t>USB2_DP</t>
+  </si>
+  <si>
+    <t>OTG2_HSDP</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>USB2 HS/FS D−</t>
+  </si>
+  <si>
+    <t>USB2_DM</t>
+  </si>
+  <si>
+    <t>OTG2_HSDM</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>Not normally needed for USB-C; retain on netlist for flexibility</t>
+  </si>
+  <si>
+    <t>USB1_ID</t>
+  </si>
+  <si>
+    <t>OTG1_ID</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>USB1_TXRTUNE</t>
+  </si>
+  <si>
+    <t>OTG1_TXRTUNE</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>CC/PD handling</t>
+  </si>
+  <si>
+    <t>Type-C CC2</t>
+  </si>
+  <si>
+    <t>USB1_CC2</t>
+  </si>
+  <si>
+    <t>UCPD1_CC2</t>
+  </si>
+  <si>
+    <t>B6</t>
+  </si>
+  <si>
+    <t>Type-C CC1</t>
+  </si>
+  <si>
+    <t>USB1_CC1</t>
+  </si>
+  <si>
+    <t>UCPD1_CC1</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>USB Type-C preferred port</t>
+  </si>
+  <si>
+    <t>USB1 HS/FS D+</t>
+  </si>
+  <si>
+    <t>USB1_DP</t>
+  </si>
+  <si>
+    <t>OTG1_HSDP</t>
+  </si>
+  <si>
+    <t>B5</t>
+  </si>
+  <si>
+    <t>USB1 HS/FS D−</t>
+  </si>
+  <si>
+    <t>USB1_DM</t>
+  </si>
+  <si>
+    <t>OTG1_HSDM</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>Use / Notes</t>
   </si>
 </sst>
 </file>
@@ -1454,6 +1921,68 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2048,61 +2577,61 @@
         <v>111</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="I21" s="3" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="I22" s="3" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2193,90 +2722,90 @@
         <v>138</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G26" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H26" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="I26" s="3" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G27" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H27" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="I27" s="3" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="G28" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="H28" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="I28" s="3" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2630,10 +3159,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3190,7 +3720,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3328,64 +3858,855 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B6"/>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA333C3D-C9BA-485C-B4F5-8B3129E6631A}">
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="43" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H17" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFEB4E61-2324-4590-A073-BA1F6E500ABB}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>413</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E4" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECA01D71-6CE0-475D-9418-AF150DFDD7D9}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="8" max="8" width="43" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>318</v>
+        <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>320</v>
+        <v>24</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>324</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>326</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>327</v>
+        <v>25</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>433</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H11" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>